<commit_message>
test: add Selenium test script and associated data file for quiz management functionality
</commit_message>
<xml_diff>
--- a/data/TC_QuizManagement.xlsx
+++ b/data/TC_QuizManagement.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC_QuizCRUD" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TC_QuizCRUD" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -804,7 +804,7 @@
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>quizzes/yY3YTi0yYJPy1IGnyJQf EXISTS (status=draft)</t>
+          <t>quizzes/SDbRehDyPxb6o2r4KqPa EXISTS (status=draft)</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:20 | Run: 2026-04-19 01:45 | Run: 2026-04-19 01:49 | Run: 2026-04-19 01:49 | Run: 2026-04-19 02:05 | Run: 2026-04-19 02:07 | Run: 2026-04-19 02:11 | Run: 2026-04-19 02:13 | Run: 2026-04-19 02:26 | Run: 2026-04-19 02:27 | Run: 2026-04-19 02:42 | Run: 2026-04-19 02:42 | Run: 2026-04-19 09:25 | Run: 2026-04-19 09:27 | Run: 2026-04-19 09:33 | Run: 2026-04-19 09:43 | Run: 2026-04-19 09:44 | Run: 2026-04-19 09:45 | Run: 2026-04-19 09:48 | Run: 2026-04-19 09:52 | Run: 2026-04-19 09:55 | Run: 2026-04-19 09:58 | Run: 2026-04-19 10:03 | Run: 2026-04-19 10:06 | Run: 2026-04-19 10:08 | Run: 2026-04-19 10:12 | Run: 2026-04-19 10:18 | Run: 2026-04-19 10:35 | Run: 2026-04-19 10:39 | Run: 2026-04-19 10:43 | Run: 2026-04-19 10:51</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:20 | Run: 2026-04-19 01:45 | Run: 2026-04-19 01:49 | Run: 2026-04-19 01:49 | Run: 2026-04-19 02:05 | Run: 2026-04-19 02:07 | Run: 2026-04-19 02:11 | Run: 2026-04-19 02:13 | Run: 2026-04-19 02:26 | Run: 2026-04-19 02:27 | Run: 2026-04-19 02:42 | Run: 2026-04-19 02:42 | Run: 2026-04-19 09:25 | Run: 2026-04-19 09:27 | Run: 2026-04-19 09:33 | Run: 2026-04-19 09:43 | Run: 2026-04-19 09:44 | Run: 2026-04-19 09:45 | Run: 2026-04-19 09:48 | Run: 2026-04-19 09:52 | Run: 2026-04-19 09:55 | Run: 2026-04-19 09:58 | Run: 2026-04-19 10:03 | Run: 2026-04-19 10:06 | Run: 2026-04-19 10:08 | Run: 2026-04-19 10:12 | Run: 2026-04-19 10:18 | Run: 2026-04-19 10:35 | Run: 2026-04-19 10:39 | Run: 2026-04-19 10:43 | Run: 2026-04-19 10:51 | Run: 2026-04-19 18:48 | Run: 2026-04-19 18:53 | Run: 2026-04-19 18:58 | Run: 2026-04-19 19:04 | Run: 2026-04-19 19:09 | Run: 2026-04-19 19:35 | Run: 2026-04-19 22:05</t>
         </is>
       </c>
     </row>
@@ -867,12 +867,12 @@
       <c r="J7" s="8" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:21 | Run: 2026-04-19 01:40 | Run: 2026-04-19 01:40 | Run: 2026-04-19 01:43 | Run: 2026-04-19 01:46 | Run: 2026-04-19 02:12 | Run: 2026-04-19 10:59 | Run: 2026-04-19 11:01</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:21 | Run: 2026-04-19 01:40 | Run: 2026-04-19 01:40 | Run: 2026-04-19 01:43 | Run: 2026-04-19 01:46 | Run: 2026-04-19 02:12 | Run: 2026-04-19 10:59 | Run: 2026-04-19 11:01 | Run: 2026-04-19 19:32 | Run: 2026-04-19 19:36</t>
         </is>
       </c>
     </row>
@@ -919,91 +919,69 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
+          <t>Continue disabled with 0 questions – validation ✓</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:21 | Run: 2026-04-19 01:46 | Run: 2026-04-19 02:12 | Run: 2026-04-19 19:38 | Run: 2026-04-19 22:34 | Run: 2026-04-19 22:41 | Run: 2026-04-19 22:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>TC-CQ-004</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Create Quiz</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Create with XSS in title</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>CREATOR</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Title='&lt;script&gt;alert(1)&lt;/script&gt;'</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Script not executed; title stored as escaped text</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Firestore stores escaped string</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Delete quiz doc</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">EXCEPTION: Message: 
 Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7a3e00245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7a3e002b0+14740]
+	chromedriver!GetHandleVerifier [0x7ff71a6e0245+146d5]
+	chromedriver!GetHandleVerifier [0x7ff71a6e02b0+14740]
 	chromedriver!(No </t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr"/>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L8" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:21 | Run: 2026-04-19 01:46 | Run: 2026-04-19 02:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>TC-CQ-004</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Create Quiz</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Create with XSS in title</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>CREATOR</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Title='&lt;script&gt;alert(1)&lt;/script&gt;'</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Script not executed; title stored as escaped text</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Firestore stores escaped string</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Delete quiz doc</t>
-        </is>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lỗi script: Message: no such element: Unable to locate element: {"method":"css selector","selector":"button[type='submit'], button.btn-login, button.login-btn"}
-  (Session info: chrome=147.0.7727.57); For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7c9380245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7c93802b0+14740]
-	chromedriver!(No symbol) [0x7ff7c90ed7cd]
-	chromedriver!(No symbol) [0x7ff7c9146c4e]
-	chromedriver!(No symbol) [0x7ff7c9146f5c]
-	chromedriver!(No symbol) [0x7ff7c9197cc7]
-	chromedriver!(No symbol) [0x7ff7c9194818]
-	chromedriver!(No symbol) [0x7ff7c9139018]
-	chromedriver!(No symbol) [0x7ff7c9139f03]
-	chromedriver!GetHandleVerifier [0x7ff7c96958f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7c968fe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7c96b30b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7c939d3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7c93a600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7c9389634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7c93897e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7c936e2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffc6910e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffc6a7ec3fc+2c]
-</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr"/>
@@ -1014,7 +992,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:21</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:21 | Run: 2026-04-19 19:41 | Run: 2026-04-19 22:53</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1039,12 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Quiz 'TC-RQ-001_Auto_1776538007': FOUND in /creator/my</t>
+          <t>Quiz 'TC-RQ-001_Auto_1776614200': FOUND in /creator/my</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>quizzes/ZT2XFN1up486obDC2Isr status=draft</t>
+          <t>quizzes/p63KyRPWdOiwlvyZhnYg status=draft</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
@@ -1076,7 +1054,7 @@
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:22 | Run: 2026-04-19 01:40 | Run: 2026-04-19 01:43 | Run: 2026-04-19 01:47</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:22 | Run: 2026-04-19 01:40 | Run: 2026-04-19 01:43 | Run: 2026-04-19 01:47 | Run: 2026-04-19 22:30 | Run: 2026-04-19 22:57</t>
         </is>
       </c>
     </row>
@@ -1123,32 +1101,14 @@
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lỗi script: Message: no such element: Unable to locate element: {"method":"css selector","selector":"button[type='submit'], button.btn-login, button.login-btn"}
-  (Session info: chrome=147.0.7727.57); For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7c9380245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7c93802b0+14740]
-	chromedriver!(No symbol) [0x7ff7c90ed7cd]
-	chromedriver!(No symbol) [0x7ff7c9146c4e]
-	chromedriver!(No symbol) [0x7ff7c9146f5c]
-	chromedriver!(No symbol) [0x7ff7c9197cc7]
-	chromedriver!(No symbol) [0x7ff7c9194818]
-	chromedriver!(No symbol) [0x7ff7c9139018]
-	chromedriver!(No symbol) [0x7ff7c9139f03]
-	chromedriver!GetHandleVerifier [0x7ff7c96958f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7c968fe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7c96b30b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7c939d3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7c93a600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7c9389634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7c93897e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7c936e2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffc6910e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffc6a7ec3fc+2c]
-</t>
-        </is>
-      </c>
-      <c r="J11" s="8" t="inlineStr"/>
+          <t>Quiz 'TC-RQ-002_Auto_1776615125' not visible in admin quiz-management</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>quizzes/IHhKms5X5rNLPFFu3JcL status=pending</t>
+        </is>
+      </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1156,7 +1116,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:22</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:22 | Run: 2026-04-19 22:59 | Run: 2026-04-19 23:04 | Run: 2026-04-19 23:08 | Run: 2026-04-19 23:13</t>
         </is>
       </c>
     </row>
@@ -1203,22 +1163,22 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>TC-CQ-001 chưa tạo quiz – skip</t>
+          <t>URL after /edit: https://datn-quizapp.web.app/quiz/MAKMl4DKaOZLOEjVyiah/edit</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>quizzes/MAKMl4DKaOZLOEjVyiah status=draft</t>
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>Bug: edit not persisted | Run: 2026-04-18 12:22</t>
+          <t>Bug: edit not persisted | Run: 2026-04-18 12:22 | Run: 2026-04-19 23:14</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1225,7 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>Không có quiz ID để test</t>
+          <t>Regular user blocked from edit page ✓</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
@@ -1275,12 +1235,12 @@
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:22</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:22 | Run: 2026-04-19 23:15</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1287,7 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Không có quiz ID để test</t>
+          <t>EXCEPTION: 403 Client Error: Forbidden for url: https://firestore.googleapis.com/v1/projects/datn-quizapp/databases/(default)/documents/quizzes</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
@@ -1337,12 +1297,12 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:22</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:22 | Run: 2026-04-19 23:16</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1364,7 @@
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>Bug: delete partially works | Run: 2026-04-18 12:22 | Run: 2026-04-19 01:47</t>
+          <t>Bug: delete partially works | Run: 2026-04-18 12:22 | Run: 2026-04-19 01:47 | Run: 2026-04-19 23:18</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1426,7 @@
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:22 | Run: 2026-04-19 01:44 | Run: 2026-04-19 01:48</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:22 | Run: 2026-04-19 01:44 | Run: 2026-04-19 01:48 | Run: 2026-04-19 23:20</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1473,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>File not found: C:\quiz-trivia-tooltest\data\sample_import_valid.csv</t>
+          <t>Import result: Chỉ chấp nhận: jpeg, png, webp</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
@@ -1523,12 +1483,12 @@
       </c>
       <c r="K17" s="9" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>Known: import fails for most formats | Run: 2026-04-18 12:22</t>
+          <t>Known: import fails for most formats | Run: 2026-04-18 12:22 | Run: 2026-04-19 23:28 | Run: 2026-04-19 23:35 | Run: 2026-04-19 23:40</t>
         </is>
       </c>
     </row>
@@ -1575,29 +1535,11 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lỗi script: Message: no such element: Unable to locate element: {"method":"css selector","selector":"button[type='submit'], button.btn-login, button.login-btn"}
-  (Session info: chrome=147.0.7727.57); For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
+          <t xml:space="preserve">EXCEPTION: Message: 
 Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7c9380245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7c93802b0+14740]
-	chromedriver!(No symbol) [0x7ff7c90ed7cd]
-	chromedriver!(No symbol) [0x7ff7c9146c4e]
-	chromedriver!(No symbol) [0x7ff7c9146f5c]
-	chromedriver!(No symbol) [0x7ff7c9197cc7]
-	chromedriver!(No symbol) [0x7ff7c9194818]
-	chromedriver!(No symbol) [0x7ff7c9139018]
-	chromedriver!(No symbol) [0x7ff7c9139f03]
-	chromedriver!GetHandleVerifier [0x7ff7c96958f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7c968fe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7c96b30b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7c939d3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7c93a600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7c9389634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7c93897e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7c936e2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffc6910e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffc6a7ec3fc+2c]
-</t>
+	chromedriver!GetHandleVerifier [0x7ff71a6e0245+146d5]
+	chromedriver!GetHandleVerifier [0x7ff71a6e02b0+14740]
+	chromedriver!(No </t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr"/>
@@ -1608,7 +1550,7 @@
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:22</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:22 | Run: 2026-04-19 23:30</t>
         </is>
       </c>
     </row>
@@ -1655,29 +1597,7 @@
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lỗi script: Message: no such element: Unable to locate element: {"method":"css selector","selector":"button[type='submit'], button.btn-login, button.login-btn"}
-  (Session info: chrome=147.0.7727.57); For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7c9380245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7c93802b0+14740]
-	chromedriver!(No symbol) [0x7ff7c90ed7cd]
-	chromedriver!(No symbol) [0x7ff7c9146c4e]
-	chromedriver!(No symbol) [0x7ff7c9146f5c]
-	chromedriver!(No symbol) [0x7ff7c9197cc7]
-	chromedriver!(No symbol) [0x7ff7c9194818]
-	chromedriver!(No symbol) [0x7ff7c9139018]
-	chromedriver!(No symbol) [0x7ff7c9139f03]
-	chromedriver!GetHandleVerifier [0x7ff7c96958f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7c968fe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7c96b30b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7c939d3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7c93a600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7c9389634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7c93897e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7c936e2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffc6910e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffc6a7ec3fc+2c]
-</t>
+          <t>Bad schema result: Chỉ chấp nhận: jpeg, png, webp</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr"/>
@@ -1688,7 +1608,7 @@
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:22</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:22 | Run: 2026-04-19 23:42</t>
         </is>
       </c>
     </row>
@@ -1735,29 +1655,7 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lỗi script: Message: no such element: Unable to locate element: {"method":"css selector","selector":"button[type='submit'], button.btn-login, button.login-btn"}
-  (Session info: chrome=147.0.7727.57); For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7c9380245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7c93802b0+14740]
-	chromedriver!(No symbol) [0x7ff7c90ed7cd]
-	chromedriver!(No symbol) [0x7ff7c9146c4e]
-	chromedriver!(No symbol) [0x7ff7c9146f5c]
-	chromedriver!(No symbol) [0x7ff7c9197cc7]
-	chromedriver!(No symbol) [0x7ff7c9194818]
-	chromedriver!(No symbol) [0x7ff7c9139018]
-	chromedriver!(No symbol) [0x7ff7c9139f03]
-	chromedriver!GetHandleVerifier [0x7ff7c96958f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7c968fe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7c96b30b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7c939d3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7c93a600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7c9389634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7c93897e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7c936e2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffc6910e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffc6a7ec3fc+2c]
-</t>
+          <t>No clear size-validation response</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr"/>
@@ -1768,7 +1666,7 @@
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:23</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:23 | Run: 2026-04-19 23:45</t>
         </is>
       </c>
     </row>
@@ -1815,22 +1713,22 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>Không có quiz ID</t>
+          <t>Draft quiz inaccessible to regular user ✓</t>
         </is>
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>quizzes/Fibt8mu2iWJNAkteCU8X status=draft</t>
         </is>
       </c>
       <c r="K21" s="10" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>Verified in system test | Run: 2026-04-18 12:23</t>
+          <t>Verified in system test | Run: 2026-04-18 12:23 | Run: 2026-04-19 23:46</t>
         </is>
       </c>
     </row>
@@ -1877,22 +1775,22 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Không có quiz ID</t>
+          <t>Submit result: No toast</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Firestore status: draft</t>
         </is>
       </c>
       <c r="K22" s="9" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>Bug: state transition unreliable | Run: 2026-04-18 12:23</t>
+          <t>Bug: state transition unreliable | Run: 2026-04-18 12:23 | Run: 2026-04-19 23:49</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1837,7 @@
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>Không có quiz ID</t>
+          <t>Quiz not found in any admin route</t>
         </is>
       </c>
       <c r="J23" s="8" t="inlineStr">
@@ -1949,12 +1847,12 @@
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>Bug: approval flow broken | Run: 2026-04-18 12:23</t>
+          <t>Bug: approval flow broken | Run: 2026-04-18 12:23 | Run: 2026-04-19 23:50</t>
         </is>
       </c>
     </row>
@@ -2001,7 +1899,7 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Không có quiz ID</t>
+          <t>EXCEPTION: 403 Client Error: Forbidden for url: https://firestore.googleapis.com/v1/projects/datn-quizapp/databases/(default)/documents/quizzes</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
@@ -2011,12 +1909,12 @@
       </c>
       <c r="K24" s="9" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>Bug: client-side only check | Run: 2026-04-18 12:23</t>
+          <t>Bug: client-side only check | Run: 2026-04-18 12:23 | Run: 2026-04-19 23:51</t>
         </is>
       </c>
     </row>
@@ -2063,7 +1961,7 @@
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Không có quiz ID</t>
+          <t>EXCEPTION: 403 Client Error: Forbidden for url: https://firestore.googleapis.com/v1/projects/datn-quizapp/databases/(default)/documents/quizzes</t>
         </is>
       </c>
       <c r="J25" s="8" t="inlineStr">
@@ -2073,12 +1971,12 @@
       </c>
       <c r="K25" s="10" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L25" s="8" t="inlineStr">
         <is>
-          <t>Verified in system test | Run: 2026-04-18 12:23</t>
+          <t>Verified in system test | Run: 2026-04-18 12:23 | Run: 2026-04-19 23:51</t>
         </is>
       </c>
     </row>
@@ -2125,40 +2023,18 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lỗi script: Message: no such element: Unable to locate element: {"method":"css selector","selector":"button[type='submit'], button.btn-login, button.login-btn"}
-  (Session info: chrome=147.0.7727.57); For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7c9380245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7c93802b0+14740]
-	chromedriver!(No symbol) [0x7ff7c90ed7cd]
-	chromedriver!(No symbol) [0x7ff7c9146c4e]
-	chromedriver!(No symbol) [0x7ff7c9146f5c]
-	chromedriver!(No symbol) [0x7ff7c9197cc7]
-	chromedriver!(No symbol) [0x7ff7c9194818]
-	chromedriver!(No symbol) [0x7ff7c9139018]
-	chromedriver!(No symbol) [0x7ff7c9139f03]
-	chromedriver!GetHandleVerifier [0x7ff7c96958f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7c968fe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7c96b30b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7c939d3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7c93a600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7c9389634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7c93897e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7c936e2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffc6910e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffc6a7ec3fc+2c]
-</t>
+          <t>dur=-1: validation blocked as expected ✓</t>
         </is>
       </c>
       <c r="J26" s="11" t="n"/>
       <c r="K26" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L26" s="11" t="inlineStr">
         <is>
-          <t>BVA: gia tri am – ngoai vung hop le | Run: 2026-04-18 12:21</t>
+          <t>BVA: gia tri am – ngoai vung hop le | Run: 2026-04-18 12:21 | Run: 2026-04-19 19:42 | Run: 2026-04-19 22:26</t>
         </is>
       </c>
     </row>
@@ -2205,40 +2081,18 @@
       </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lỗi script: Message: no such element: Unable to locate element: {"method":"css selector","selector":"button[type='submit'], button.btn-login, button.login-btn"}
-  (Session info: chrome=147.0.7727.57); For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7c9380245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7c93802b0+14740]
-	chromedriver!(No symbol) [0x7ff7c90ed7cd]
-	chromedriver!(No symbol) [0x7ff7c9146c4e]
-	chromedriver!(No symbol) [0x7ff7c9146f5c]
-	chromedriver!(No symbol) [0x7ff7c9197cc7]
-	chromedriver!(No symbol) [0x7ff7c9194818]
-	chromedriver!(No symbol) [0x7ff7c9139018]
-	chromedriver!(No symbol) [0x7ff7c9139f03]
-	chromedriver!GetHandleVerifier [0x7ff7c96958f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7c968fe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7c96b30b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7c939d3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7c93a600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7c9389634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7c93897e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7c936e2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffc6910e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffc6a7ec3fc+2c]
-</t>
+          <t>dur=4: validation blocked as expected ✓</t>
         </is>
       </c>
       <c r="J27" s="11" t="n"/>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L27" s="11" t="inlineStr">
         <is>
-          <t>BVA: bien duoi - 1 = 4 (invalid) | Run: 2026-04-18 12:21</t>
+          <t>BVA: bien duoi - 1 = 4 (invalid) | Run: 2026-04-18 12:21 | Run: 2026-04-19 19:44 | Run: 2026-04-19 22:28</t>
         </is>
       </c>
     </row>
@@ -2285,29 +2139,7 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lỗi script: Message: no such element: Unable to locate element: {"method":"css selector","selector":"button[type='submit'], button.btn-login, button.login-btn"}
-  (Session info: chrome=147.0.7727.57); For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7c9380245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7c93802b0+14740]
-	chromedriver!(No symbol) [0x7ff7c90ed7cd]
-	chromedriver!(No symbol) [0x7ff7c9146c4e]
-	chromedriver!(No symbol) [0x7ff7c9146f5c]
-	chromedriver!(No symbol) [0x7ff7c9197cc7]
-	chromedriver!(No symbol) [0x7ff7c9194818]
-	chromedriver!(No symbol) [0x7ff7c9139018]
-	chromedriver!(No symbol) [0x7ff7c9139f03]
-	chromedriver!GetHandleVerifier [0x7ff7c96958f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7c968fe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7c96b30b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7c939d3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7c93a600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7c9389634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7c93897e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7c936e2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffc6910e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffc6a7ec3fc+2c]
-</t>
+          <t>dur=5: did not advance to Questions step</t>
         </is>
       </c>
       <c r="J28" s="11" t="n"/>
@@ -2318,7 +2150,7 @@
       </c>
       <c r="L28" s="11" t="inlineStr">
         <is>
-          <t>BVA: bien duoi = 5 (valid) | Run: 2026-04-18 12:21</t>
+          <t>BVA: bien duoi = 5 (valid) | Run: 2026-04-18 12:21 | Run: 2026-04-19 19:47</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2167,7 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Duration = 6 (bien duoi + 1) phai duoc chap nhan</t>
+          <t>Duration = 120 (bien tren) phai duoc chap nhan</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
@@ -2345,7 +2177,7 @@
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>Title='Test Quiz BVA'; thong tin hop le; Duration = 6</t>
+          <t>Title='Test Quiz BVA'; thong tin hop le; Duration = 120</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
@@ -2355,7 +2187,7 @@
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
-          <t>Quiz doc duoc tao trong Firestore voi duration = 6</t>
+          <t>Quiz doc duoc tao trong Firestore voi duration = 120</t>
         </is>
       </c>
       <c r="H29" s="11" t="inlineStr">
@@ -2363,16 +2195,20 @@
           <t>Xoa quiz doc via Firestore REST API</t>
         </is>
       </c>
-      <c r="I29" s="11" t="n"/>
+      <c r="I29" s="11" t="inlineStr">
+        <is>
+          <t>dur=120: did not advance to Questions step</t>
+        </is>
+      </c>
       <c r="J29" s="11" t="n"/>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L29" s="11" t="inlineStr">
         <is>
-          <t>BVA: bien duoi + 1 = 6 (valid)</t>
+          <t>BVA: bien tren = 120 (valid) | Run: 2026-04-18 12:22 | Run: 2026-04-19 21:42 | Run: 2026-04-19 22:08</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2225,7 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Duration = 119 (bien tren - 1) phai duoc chap nhan</t>
+          <t>Duration = 121 (bien tren + 1) phai bi tu choi</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2399,197 +2235,43 @@
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Title='Test Quiz BVA'; thong tin hop le; Duration = 119</t>
+          <t>Title='Test Quiz BVA'; thong tin hop le; Duration = 121</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>Chuyen sang buoc tiep theo thanh cong; khong co loi</t>
+          <t>Hien thi loi hoac button Next bi disabled; khong chuyen buoc</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Quiz doc duoc tao trong Firestore voi duration = 119</t>
+          <t>Khong co document nao duoc tao trong Firestore</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>Xoa quiz doc via Firestore REST API</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="n"/>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>dur=121: validation blocked as expected ✓</t>
+        </is>
+      </c>
       <c r="J30" s="11" t="n"/>
       <c r="K30" s="11" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L30" s="11" t="inlineStr">
         <is>
-          <t>BVA: bien tren - 1 = 119 (valid)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="55" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>TC-CQ-010</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>Create Quiz - Duration</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>Duration = 120 (bien tren) phai duoc chap nhan</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>CREATOR</t>
-        </is>
-      </c>
-      <c r="E31" s="11" t="inlineStr">
-        <is>
-          <t>Title='Test Quiz BVA'; thong tin hop le; Duration = 120</t>
-        </is>
-      </c>
-      <c r="F31" s="11" t="inlineStr">
-        <is>
-          <t>Chuyen sang buoc tiep theo thanh cong; khong co loi</t>
-        </is>
-      </c>
-      <c r="G31" s="11" t="inlineStr">
-        <is>
-          <t>Quiz doc duoc tao trong Firestore voi duration = 120</t>
-        </is>
-      </c>
-      <c r="H31" s="11" t="inlineStr">
-        <is>
-          <t>Xoa quiz doc via Firestore REST API</t>
-        </is>
-      </c>
-      <c r="I31" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lỗi script: Message: no such element: Unable to locate element: {"method":"css selector","selector":"button[type='submit'], button.btn-login, button.login-btn"}
-  (Session info: chrome=147.0.7727.57); For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7c9380245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7c93802b0+14740]
-	chromedriver!(No symbol) [0x7ff7c90ed7cd]
-	chromedriver!(No symbol) [0x7ff7c9146c4e]
-	chromedriver!(No symbol) [0x7ff7c9146f5c]
-	chromedriver!(No symbol) [0x7ff7c9197cc7]
-	chromedriver!(No symbol) [0x7ff7c9194818]
-	chromedriver!(No symbol) [0x7ff7c9139018]
-	chromedriver!(No symbol) [0x7ff7c9139f03]
-	chromedriver!GetHandleVerifier [0x7ff7c96958f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7c968fe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7c96b30b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7c939d3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7c93a600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7c9389634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7c93897e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7c936e2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffc6910e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffc6a7ec3fc+2c]
-</t>
-        </is>
-      </c>
-      <c r="J31" s="11" t="n"/>
-      <c r="K31" s="11" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L31" s="11" t="inlineStr">
-        <is>
-          <t>BVA: bien tren = 120 (valid) | Run: 2026-04-18 12:22</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="55" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>TC-CQ-011</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>Create Quiz - Duration</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>Duration = 121 (bien tren + 1) phai bi tu choi</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>CREATOR</t>
-        </is>
-      </c>
-      <c r="E32" s="11" t="inlineStr">
-        <is>
-          <t>Title='Test Quiz BVA'; thong tin hop le; Duration = 121</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>Hien thi loi hoac button Next bi disabled; khong chuyen buoc</t>
-        </is>
-      </c>
-      <c r="G32" s="11" t="inlineStr">
-        <is>
-          <t>Khong co document nao duoc tao trong Firestore</t>
-        </is>
-      </c>
-      <c r="H32" s="11" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lỗi script: Message: no such element: Unable to locate element: {"method":"css selector","selector":"button[type='submit'], button.btn-login, button.login-btn"}
-  (Session info: chrome=147.0.7727.57); For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff7c9380245+146d5]
-	chromedriver!GetHandleVerifier [0x7ff7c93802b0+14740]
-	chromedriver!(No symbol) [0x7ff7c90ed7cd]
-	chromedriver!(No symbol) [0x7ff7c9146c4e]
-	chromedriver!(No symbol) [0x7ff7c9146f5c]
-	chromedriver!(No symbol) [0x7ff7c9197cc7]
-	chromedriver!(No symbol) [0x7ff7c9194818]
-	chromedriver!(No symbol) [0x7ff7c9139018]
-	chromedriver!(No symbol) [0x7ff7c9139f03]
-	chromedriver!GetHandleVerifier [0x7ff7c96958f9+329d89]
-	chromedriver!GetHandleVerifier [0x7ff7c968fe46+3242d6]
-	chromedriver!GetHandleVerifier [0x7ff7c96b30b2+347542]
-	chromedriver!GetHandleVerifier [0x7ff7c939d3d5+31865]
-	chromedriver!GetHandleVerifier [0x7ff7c93a600c+3a49c]
-	chromedriver!GetHandleVerifier [0x7ff7c9389634+1dac4]
-	chromedriver!GetHandleVerifier [0x7ff7c93897e6+1dc76]
-	chromedriver!GetHandleVerifier [0x7ff7c936e2f7+2787]
-	KERNEL32!BaseThreadInitThunk [0x7ffc6910e8d7+17]
-	ntdll!RtlUserThreadStart [0x7ffc6a7ec3fc+2c]
-</t>
-        </is>
-      </c>
-      <c r="J32" s="11" t="n"/>
-      <c r="K32" s="11" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L32" s="11" t="inlineStr">
-        <is>
-          <t>BVA: bien tren + 1 = 121 (invalid) | Run: 2026-04-18 12:22</t>
-        </is>
-      </c>
-    </row>
+          <t>BVA: bien tren + 1 = 121 (invalid) | Run: 2026-04-18 12:22 | Run: 2026-04-19 22:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="55" customHeight="1"/>
+    <row r="32" ht="55" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:L2"/>

</xml_diff>